<commit_message>
Template SPEC: ae_overview, with its sample report in the onco example
The onco example study gains T-14-3-2, Overview of Treatment-Emergent
Adverse Events (make_specs.R and its three table workbooks; the other
tables' programs and RTF unchanged). The display template ae_overview on
summary (tpl_ae_overview()): a subjects analysis a row (any, related,
grade 3+, serious, leading to discontinuation, leading to death), one row
a flag (no label column). Same items and RTF by the spec, by B and by A.
0.0.24.9155. Closes #335.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/examples/onco/spec/ard_spec.xlsx
+++ b/inst/examples/onco/spec/ard_spec.xlsx
@@ -638,7 +638,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="109">
   <si>
     <t xml:space="preserve">key</t>
   </si>
@@ -769,6 +769,18 @@
     <t xml:space="preserve">TRTEMFL == "Y"</t>
   </si>
   <si>
+    <t xml:space="preserve">T-14-3-2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">adsl_saf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Safety set</t>
+  </si>
+  <si>
+    <t xml:space="preserve">adae_saf</t>
+  </si>
+  <si>
     <t xml:space="preserve">analysis_id</t>
   </si>
   <si>
@@ -896,6 +908,63 @@
   </si>
   <si>
     <t xml:space="preserve">over_variables = TRUE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GROUPN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PRIMARY OUTCOME MEASURE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Any TEAE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Any treatment-related TEAE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AEREL == "RELATED"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Any TEAE of CTCAE grade 3 or higher</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AETOXGR %in% c("3", "4", "5")</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Any serious TEAE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AESER == "Y"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DISC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Any TEAE leading to discontinuation of study drug</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AEACN == "DRUG WITHDRAWN"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DTH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Any TEAE leading to death</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AEOUT == "FATAL"</t>
   </si>
 </sst>
 </file>
@@ -1473,6 +1542,54 @@
       <c r="K3"/>
       <c r="L3"/>
     </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4"/>
+      <c r="G4"/>
+      <c r="H4"/>
+      <c r="I4"/>
+      <c r="J4"/>
+      <c r="K4"/>
+      <c r="L4"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C5"/>
+      <c r="D5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5"/>
+      <c r="F5" t="s">
+        <v>44</v>
+      </c>
+      <c r="G5" t="s">
+        <v>42</v>
+      </c>
+      <c r="H5"/>
+      <c r="I5"/>
+      <c r="J5"/>
+      <c r="K5"/>
+      <c r="L5"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
@@ -1490,19 +1607,19 @@
         <v>26</v>
       </c>
       <c r="B1" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C1" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="D1" t="s">
         <v>19</v>
       </c>
       <c r="E1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="F1" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="G1" t="s">
         <v>6</v>
@@ -1514,55 +1631,55 @@
         <v>18</v>
       </c>
       <c r="J1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="K1" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="L1" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="M1" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="N1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="O1" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="P1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="Q1" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="R1" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="S1" t="s">
         <v>33</v>
       </c>
       <c r="T1" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="U1" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B2" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C2"/>
       <c r="D2" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="E2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="F2"/>
       <c r="G2"/>
@@ -1574,7 +1691,7 @@
       <c r="K2"/>
       <c r="L2"/>
       <c r="M2" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="N2"/>
       <c r="O2"/>
@@ -1587,17 +1704,17 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B3" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C3"/>
       <c r="D3" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E3" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="F3"/>
       <c r="G3"/>
@@ -1606,12 +1723,12 @@
       </c>
       <c r="I3"/>
       <c r="J3" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="K3"/>
       <c r="L3"/>
       <c r="M3" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="N3"/>
       <c r="O3"/>
@@ -1624,17 +1741,17 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B4" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C4"/>
       <c r="D4" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E4" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="F4"/>
       <c r="G4"/>
@@ -1643,12 +1760,12 @@
       </c>
       <c r="I4"/>
       <c r="J4" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="K4"/>
       <c r="L4"/>
       <c r="M4" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="N4"/>
       <c r="O4"/>
@@ -1664,14 +1781,14 @@
         <v>34</v>
       </c>
       <c r="B5" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C5"/>
       <c r="D5" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="E5" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="F5"/>
       <c r="G5"/>
@@ -1683,7 +1800,7 @@
       <c r="K5"/>
       <c r="L5"/>
       <c r="M5" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="N5"/>
       <c r="O5"/>
@@ -1699,14 +1816,14 @@
         <v>34</v>
       </c>
       <c r="B6" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C6"/>
       <c r="D6" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="E6" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="F6" t="s">
         <v>35</v>
@@ -1715,12 +1832,12 @@
       <c r="H6"/>
       <c r="I6"/>
       <c r="J6" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="K6"/>
       <c r="L6"/>
       <c r="M6" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="N6"/>
       <c r="O6"/>
@@ -1736,14 +1853,14 @@
         <v>34</v>
       </c>
       <c r="B7" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C7"/>
       <c r="D7" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="E7" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F7" t="s">
         <v>35</v>
@@ -1752,18 +1869,18 @@
       <c r="H7"/>
       <c r="I7"/>
       <c r="J7" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="K7"/>
       <c r="L7"/>
       <c r="M7" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="N7"/>
       <c r="O7"/>
       <c r="P7"/>
       <c r="Q7" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="R7"/>
       <c r="S7"/>
@@ -1775,14 +1892,14 @@
         <v>34</v>
       </c>
       <c r="B8" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C8"/>
       <c r="D8" t="s">
+        <v>84</v>
+      </c>
+      <c r="E8" t="s">
         <v>80</v>
-      </c>
-      <c r="E8" t="s">
-        <v>76</v>
       </c>
       <c r="F8" t="s">
         <v>35</v>
@@ -1791,18 +1908,18 @@
       <c r="H8"/>
       <c r="I8"/>
       <c r="J8" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="K8"/>
       <c r="L8"/>
       <c r="M8" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="N8"/>
       <c r="O8"/>
       <c r="P8"/>
       <c r="Q8" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="R8"/>
       <c r="S8"/>
@@ -1814,14 +1931,14 @@
         <v>39</v>
       </c>
       <c r="B9" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C9"/>
       <c r="D9" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="E9" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="F9"/>
       <c r="G9"/>
@@ -1833,7 +1950,7 @@
       <c r="K9"/>
       <c r="L9"/>
       <c r="M9" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="N9"/>
       <c r="O9"/>
@@ -1849,14 +1966,14 @@
         <v>39</v>
       </c>
       <c r="B10" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="C10"/>
       <c r="D10" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="E10" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="F10" t="s">
         <v>40</v>
@@ -1865,12 +1982,12 @@
       <c r="H10"/>
       <c r="I10"/>
       <c r="J10" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="K10"/>
       <c r="L10"/>
       <c r="M10" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="N10"/>
       <c r="O10" t="s">
@@ -1878,12 +1995,291 @@
       </c>
       <c r="P10"/>
       <c r="Q10" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="R10"/>
       <c r="S10"/>
       <c r="T10"/>
       <c r="U10"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B11" t="s">
+        <v>90</v>
+      </c>
+      <c r="C11"/>
+      <c r="D11"/>
+      <c r="E11" t="s">
+        <v>65</v>
+      </c>
+      <c r="F11" t="s">
+        <v>44</v>
+      </c>
+      <c r="G11"/>
+      <c r="H11"/>
+      <c r="I11"/>
+      <c r="J11"/>
+      <c r="K11"/>
+      <c r="L11"/>
+      <c r="M11" t="s">
+        <v>66</v>
+      </c>
+      <c r="N11"/>
+      <c r="O11"/>
+      <c r="P11"/>
+      <c r="Q11"/>
+      <c r="R11"/>
+      <c r="S11"/>
+      <c r="T11" t="s">
+        <v>91</v>
+      </c>
+      <c r="U11"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>43</v>
+      </c>
+      <c r="B12" t="s">
+        <v>92</v>
+      </c>
+      <c r="C12"/>
+      <c r="D12" t="s">
+        <v>93</v>
+      </c>
+      <c r="E12" t="s">
+        <v>29</v>
+      </c>
+      <c r="F12" t="s">
+        <v>46</v>
+      </c>
+      <c r="G12"/>
+      <c r="H12"/>
+      <c r="I12"/>
+      <c r="J12" t="s">
+        <v>66</v>
+      </c>
+      <c r="K12"/>
+      <c r="L12"/>
+      <c r="M12" t="s">
+        <v>92</v>
+      </c>
+      <c r="N12"/>
+      <c r="O12"/>
+      <c r="P12"/>
+      <c r="Q12"/>
+      <c r="R12"/>
+      <c r="S12"/>
+      <c r="T12" t="s">
+        <v>91</v>
+      </c>
+      <c r="U12"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B13" t="s">
+        <v>94</v>
+      </c>
+      <c r="C13"/>
+      <c r="D13" t="s">
+        <v>95</v>
+      </c>
+      <c r="E13" t="s">
+        <v>29</v>
+      </c>
+      <c r="F13" t="s">
+        <v>46</v>
+      </c>
+      <c r="G13"/>
+      <c r="H13"/>
+      <c r="I13" t="s">
+        <v>96</v>
+      </c>
+      <c r="J13" t="s">
+        <v>66</v>
+      </c>
+      <c r="K13"/>
+      <c r="L13"/>
+      <c r="M13" t="s">
+        <v>94</v>
+      </c>
+      <c r="N13"/>
+      <c r="O13"/>
+      <c r="P13"/>
+      <c r="Q13"/>
+      <c r="R13"/>
+      <c r="S13"/>
+      <c r="T13" t="s">
+        <v>91</v>
+      </c>
+      <c r="U13"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B14" t="s">
+        <v>97</v>
+      </c>
+      <c r="C14"/>
+      <c r="D14" t="s">
+        <v>98</v>
+      </c>
+      <c r="E14" t="s">
+        <v>29</v>
+      </c>
+      <c r="F14" t="s">
+        <v>46</v>
+      </c>
+      <c r="G14"/>
+      <c r="H14"/>
+      <c r="I14" t="s">
+        <v>99</v>
+      </c>
+      <c r="J14" t="s">
+        <v>66</v>
+      </c>
+      <c r="K14"/>
+      <c r="L14"/>
+      <c r="M14" t="s">
+        <v>97</v>
+      </c>
+      <c r="N14"/>
+      <c r="O14"/>
+      <c r="P14"/>
+      <c r="Q14"/>
+      <c r="R14"/>
+      <c r="S14"/>
+      <c r="T14" t="s">
+        <v>91</v>
+      </c>
+      <c r="U14"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>43</v>
+      </c>
+      <c r="B15" t="s">
+        <v>100</v>
+      </c>
+      <c r="C15"/>
+      <c r="D15" t="s">
+        <v>101</v>
+      </c>
+      <c r="E15" t="s">
+        <v>29</v>
+      </c>
+      <c r="F15" t="s">
+        <v>46</v>
+      </c>
+      <c r="G15"/>
+      <c r="H15"/>
+      <c r="I15" t="s">
+        <v>102</v>
+      </c>
+      <c r="J15" t="s">
+        <v>66</v>
+      </c>
+      <c r="K15"/>
+      <c r="L15"/>
+      <c r="M15" t="s">
+        <v>100</v>
+      </c>
+      <c r="N15"/>
+      <c r="O15"/>
+      <c r="P15"/>
+      <c r="Q15"/>
+      <c r="R15"/>
+      <c r="S15"/>
+      <c r="T15" t="s">
+        <v>91</v>
+      </c>
+      <c r="U15"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>43</v>
+      </c>
+      <c r="B16" t="s">
+        <v>103</v>
+      </c>
+      <c r="C16"/>
+      <c r="D16" t="s">
+        <v>104</v>
+      </c>
+      <c r="E16" t="s">
+        <v>29</v>
+      </c>
+      <c r="F16" t="s">
+        <v>46</v>
+      </c>
+      <c r="G16"/>
+      <c r="H16"/>
+      <c r="I16" t="s">
+        <v>105</v>
+      </c>
+      <c r="J16" t="s">
+        <v>66</v>
+      </c>
+      <c r="K16"/>
+      <c r="L16"/>
+      <c r="M16" t="s">
+        <v>103</v>
+      </c>
+      <c r="N16"/>
+      <c r="O16"/>
+      <c r="P16"/>
+      <c r="Q16"/>
+      <c r="R16"/>
+      <c r="S16"/>
+      <c r="T16" t="s">
+        <v>91</v>
+      </c>
+      <c r="U16"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>43</v>
+      </c>
+      <c r="B17" t="s">
+        <v>106</v>
+      </c>
+      <c r="C17"/>
+      <c r="D17" t="s">
+        <v>107</v>
+      </c>
+      <c r="E17" t="s">
+        <v>29</v>
+      </c>
+      <c r="F17" t="s">
+        <v>46</v>
+      </c>
+      <c r="G17"/>
+      <c r="H17"/>
+      <c r="I17" t="s">
+        <v>108</v>
+      </c>
+      <c r="J17" t="s">
+        <v>66</v>
+      </c>
+      <c r="K17"/>
+      <c r="L17"/>
+      <c r="M17" t="s">
+        <v>106</v>
+      </c>
+      <c r="N17"/>
+      <c r="O17"/>
+      <c r="P17"/>
+      <c r="Q17"/>
+      <c r="R17"/>
+      <c r="S17"/>
+      <c r="T17" t="s">
+        <v>91</v>
+      </c>
+      <c r="U17"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Template SPEC: ae_overview, with its sample report in the onco example (#336)
The onco example study gains T-14-3-2, Overview of Treatment-Emergent
Adverse Events (make_specs.R and its three table workbooks; the other
tables' programs and RTF unchanged). The display template ae_overview on
summary (tpl_ae_overview()): a subjects analysis a row (any, related,
grade 3+, serious, leading to discontinuation, leading to death), one row
a flag (no label column). Same items and RTF by the spec, by B and by A.
0.0.24.9155. Closes #335.

Co-authored-by: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/examples/onco/spec/ard_spec.xlsx
+++ b/inst/examples/onco/spec/ard_spec.xlsx
@@ -638,7 +638,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="109">
   <si>
     <t xml:space="preserve">key</t>
   </si>
@@ -769,6 +769,18 @@
     <t xml:space="preserve">TRTEMFL == "Y"</t>
   </si>
   <si>
+    <t xml:space="preserve">T-14-3-2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">adsl_saf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Safety set</t>
+  </si>
+  <si>
+    <t xml:space="preserve">adae_saf</t>
+  </si>
+  <si>
     <t xml:space="preserve">analysis_id</t>
   </si>
   <si>
@@ -896,6 +908,63 @@
   </si>
   <si>
     <t xml:space="preserve">over_variables = TRUE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GROUPN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PRIMARY OUTCOME MEASURE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Any TEAE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Any treatment-related TEAE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AEREL == "RELATED"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Any TEAE of CTCAE grade 3 or higher</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AETOXGR %in% c("3", "4", "5")</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Any serious TEAE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AESER == "Y"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DISC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Any TEAE leading to discontinuation of study drug</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AEACN == "DRUG WITHDRAWN"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DTH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Any TEAE leading to death</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AEOUT == "FATAL"</t>
   </si>
 </sst>
 </file>
@@ -1473,6 +1542,54 @@
       <c r="K3"/>
       <c r="L3"/>
     </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4"/>
+      <c r="G4"/>
+      <c r="H4"/>
+      <c r="I4"/>
+      <c r="J4"/>
+      <c r="K4"/>
+      <c r="L4"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C5"/>
+      <c r="D5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5"/>
+      <c r="F5" t="s">
+        <v>44</v>
+      </c>
+      <c r="G5" t="s">
+        <v>42</v>
+      </c>
+      <c r="H5"/>
+      <c r="I5"/>
+      <c r="J5"/>
+      <c r="K5"/>
+      <c r="L5"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
@@ -1490,19 +1607,19 @@
         <v>26</v>
       </c>
       <c r="B1" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C1" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="D1" t="s">
         <v>19</v>
       </c>
       <c r="E1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="F1" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="G1" t="s">
         <v>6</v>
@@ -1514,55 +1631,55 @@
         <v>18</v>
       </c>
       <c r="J1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="K1" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="L1" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="M1" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="N1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="O1" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="P1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="Q1" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="R1" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="S1" t="s">
         <v>33</v>
       </c>
       <c r="T1" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="U1" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B2" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C2"/>
       <c r="D2" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="E2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="F2"/>
       <c r="G2"/>
@@ -1574,7 +1691,7 @@
       <c r="K2"/>
       <c r="L2"/>
       <c r="M2" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="N2"/>
       <c r="O2"/>
@@ -1587,17 +1704,17 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B3" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C3"/>
       <c r="D3" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E3" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="F3"/>
       <c r="G3"/>
@@ -1606,12 +1723,12 @@
       </c>
       <c r="I3"/>
       <c r="J3" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="K3"/>
       <c r="L3"/>
       <c r="M3" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="N3"/>
       <c r="O3"/>
@@ -1624,17 +1741,17 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B4" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C4"/>
       <c r="D4" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E4" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="F4"/>
       <c r="G4"/>
@@ -1643,12 +1760,12 @@
       </c>
       <c r="I4"/>
       <c r="J4" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="K4"/>
       <c r="L4"/>
       <c r="M4" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="N4"/>
       <c r="O4"/>
@@ -1664,14 +1781,14 @@
         <v>34</v>
       </c>
       <c r="B5" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C5"/>
       <c r="D5" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="E5" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="F5"/>
       <c r="G5"/>
@@ -1683,7 +1800,7 @@
       <c r="K5"/>
       <c r="L5"/>
       <c r="M5" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="N5"/>
       <c r="O5"/>
@@ -1699,14 +1816,14 @@
         <v>34</v>
       </c>
       <c r="B6" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C6"/>
       <c r="D6" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="E6" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="F6" t="s">
         <v>35</v>
@@ -1715,12 +1832,12 @@
       <c r="H6"/>
       <c r="I6"/>
       <c r="J6" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="K6"/>
       <c r="L6"/>
       <c r="M6" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="N6"/>
       <c r="O6"/>
@@ -1736,14 +1853,14 @@
         <v>34</v>
       </c>
       <c r="B7" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C7"/>
       <c r="D7" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="E7" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F7" t="s">
         <v>35</v>
@@ -1752,18 +1869,18 @@
       <c r="H7"/>
       <c r="I7"/>
       <c r="J7" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="K7"/>
       <c r="L7"/>
       <c r="M7" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="N7"/>
       <c r="O7"/>
       <c r="P7"/>
       <c r="Q7" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="R7"/>
       <c r="S7"/>
@@ -1775,14 +1892,14 @@
         <v>34</v>
       </c>
       <c r="B8" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C8"/>
       <c r="D8" t="s">
+        <v>84</v>
+      </c>
+      <c r="E8" t="s">
         <v>80</v>
-      </c>
-      <c r="E8" t="s">
-        <v>76</v>
       </c>
       <c r="F8" t="s">
         <v>35</v>
@@ -1791,18 +1908,18 @@
       <c r="H8"/>
       <c r="I8"/>
       <c r="J8" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="K8"/>
       <c r="L8"/>
       <c r="M8" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="N8"/>
       <c r="O8"/>
       <c r="P8"/>
       <c r="Q8" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="R8"/>
       <c r="S8"/>
@@ -1814,14 +1931,14 @@
         <v>39</v>
       </c>
       <c r="B9" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C9"/>
       <c r="D9" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="E9" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="F9"/>
       <c r="G9"/>
@@ -1833,7 +1950,7 @@
       <c r="K9"/>
       <c r="L9"/>
       <c r="M9" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="N9"/>
       <c r="O9"/>
@@ -1849,14 +1966,14 @@
         <v>39</v>
       </c>
       <c r="B10" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="C10"/>
       <c r="D10" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="E10" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="F10" t="s">
         <v>40</v>
@@ -1865,12 +1982,12 @@
       <c r="H10"/>
       <c r="I10"/>
       <c r="J10" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="K10"/>
       <c r="L10"/>
       <c r="M10" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="N10"/>
       <c r="O10" t="s">
@@ -1878,12 +1995,291 @@
       </c>
       <c r="P10"/>
       <c r="Q10" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="R10"/>
       <c r="S10"/>
       <c r="T10"/>
       <c r="U10"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B11" t="s">
+        <v>90</v>
+      </c>
+      <c r="C11"/>
+      <c r="D11"/>
+      <c r="E11" t="s">
+        <v>65</v>
+      </c>
+      <c r="F11" t="s">
+        <v>44</v>
+      </c>
+      <c r="G11"/>
+      <c r="H11"/>
+      <c r="I11"/>
+      <c r="J11"/>
+      <c r="K11"/>
+      <c r="L11"/>
+      <c r="M11" t="s">
+        <v>66</v>
+      </c>
+      <c r="N11"/>
+      <c r="O11"/>
+      <c r="P11"/>
+      <c r="Q11"/>
+      <c r="R11"/>
+      <c r="S11"/>
+      <c r="T11" t="s">
+        <v>91</v>
+      </c>
+      <c r="U11"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>43</v>
+      </c>
+      <c r="B12" t="s">
+        <v>92</v>
+      </c>
+      <c r="C12"/>
+      <c r="D12" t="s">
+        <v>93</v>
+      </c>
+      <c r="E12" t="s">
+        <v>29</v>
+      </c>
+      <c r="F12" t="s">
+        <v>46</v>
+      </c>
+      <c r="G12"/>
+      <c r="H12"/>
+      <c r="I12"/>
+      <c r="J12" t="s">
+        <v>66</v>
+      </c>
+      <c r="K12"/>
+      <c r="L12"/>
+      <c r="M12" t="s">
+        <v>92</v>
+      </c>
+      <c r="N12"/>
+      <c r="O12"/>
+      <c r="P12"/>
+      <c r="Q12"/>
+      <c r="R12"/>
+      <c r="S12"/>
+      <c r="T12" t="s">
+        <v>91</v>
+      </c>
+      <c r="U12"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B13" t="s">
+        <v>94</v>
+      </c>
+      <c r="C13"/>
+      <c r="D13" t="s">
+        <v>95</v>
+      </c>
+      <c r="E13" t="s">
+        <v>29</v>
+      </c>
+      <c r="F13" t="s">
+        <v>46</v>
+      </c>
+      <c r="G13"/>
+      <c r="H13"/>
+      <c r="I13" t="s">
+        <v>96</v>
+      </c>
+      <c r="J13" t="s">
+        <v>66</v>
+      </c>
+      <c r="K13"/>
+      <c r="L13"/>
+      <c r="M13" t="s">
+        <v>94</v>
+      </c>
+      <c r="N13"/>
+      <c r="O13"/>
+      <c r="P13"/>
+      <c r="Q13"/>
+      <c r="R13"/>
+      <c r="S13"/>
+      <c r="T13" t="s">
+        <v>91</v>
+      </c>
+      <c r="U13"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B14" t="s">
+        <v>97</v>
+      </c>
+      <c r="C14"/>
+      <c r="D14" t="s">
+        <v>98</v>
+      </c>
+      <c r="E14" t="s">
+        <v>29</v>
+      </c>
+      <c r="F14" t="s">
+        <v>46</v>
+      </c>
+      <c r="G14"/>
+      <c r="H14"/>
+      <c r="I14" t="s">
+        <v>99</v>
+      </c>
+      <c r="J14" t="s">
+        <v>66</v>
+      </c>
+      <c r="K14"/>
+      <c r="L14"/>
+      <c r="M14" t="s">
+        <v>97</v>
+      </c>
+      <c r="N14"/>
+      <c r="O14"/>
+      <c r="P14"/>
+      <c r="Q14"/>
+      <c r="R14"/>
+      <c r="S14"/>
+      <c r="T14" t="s">
+        <v>91</v>
+      </c>
+      <c r="U14"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>43</v>
+      </c>
+      <c r="B15" t="s">
+        <v>100</v>
+      </c>
+      <c r="C15"/>
+      <c r="D15" t="s">
+        <v>101</v>
+      </c>
+      <c r="E15" t="s">
+        <v>29</v>
+      </c>
+      <c r="F15" t="s">
+        <v>46</v>
+      </c>
+      <c r="G15"/>
+      <c r="H15"/>
+      <c r="I15" t="s">
+        <v>102</v>
+      </c>
+      <c r="J15" t="s">
+        <v>66</v>
+      </c>
+      <c r="K15"/>
+      <c r="L15"/>
+      <c r="M15" t="s">
+        <v>100</v>
+      </c>
+      <c r="N15"/>
+      <c r="O15"/>
+      <c r="P15"/>
+      <c r="Q15"/>
+      <c r="R15"/>
+      <c r="S15"/>
+      <c r="T15" t="s">
+        <v>91</v>
+      </c>
+      <c r="U15"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>43</v>
+      </c>
+      <c r="B16" t="s">
+        <v>103</v>
+      </c>
+      <c r="C16"/>
+      <c r="D16" t="s">
+        <v>104</v>
+      </c>
+      <c r="E16" t="s">
+        <v>29</v>
+      </c>
+      <c r="F16" t="s">
+        <v>46</v>
+      </c>
+      <c r="G16"/>
+      <c r="H16"/>
+      <c r="I16" t="s">
+        <v>105</v>
+      </c>
+      <c r="J16" t="s">
+        <v>66</v>
+      </c>
+      <c r="K16"/>
+      <c r="L16"/>
+      <c r="M16" t="s">
+        <v>103</v>
+      </c>
+      <c r="N16"/>
+      <c r="O16"/>
+      <c r="P16"/>
+      <c r="Q16"/>
+      <c r="R16"/>
+      <c r="S16"/>
+      <c r="T16" t="s">
+        <v>91</v>
+      </c>
+      <c r="U16"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>43</v>
+      </c>
+      <c r="B17" t="s">
+        <v>106</v>
+      </c>
+      <c r="C17"/>
+      <c r="D17" t="s">
+        <v>107</v>
+      </c>
+      <c r="E17" t="s">
+        <v>29</v>
+      </c>
+      <c r="F17" t="s">
+        <v>46</v>
+      </c>
+      <c r="G17"/>
+      <c r="H17"/>
+      <c r="I17" t="s">
+        <v>108</v>
+      </c>
+      <c r="J17" t="s">
+        <v>66</v>
+      </c>
+      <c r="K17"/>
+      <c r="L17"/>
+      <c r="M17" t="s">
+        <v>106</v>
+      </c>
+      <c r="N17"/>
+      <c r="O17"/>
+      <c r="P17"/>
+      <c r="Q17"/>
+      <c r="R17"/>
+      <c r="S17"/>
+      <c r="T17" t="s">
+        <v>91</v>
+      </c>
+      <c r="U17"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>